<commit_message>
Fix bug, pzword pzpng pzjpg pzzip pzexcel webpdf,Fix ORM mysql pg sqlite
</commit_message>
<xml_diff>
--- a/docs/kk_out.xlsx
+++ b/docs/kk_out.xlsx
@@ -26,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -63,23 +63,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -94,15 +91,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="1" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -296,7 +296,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -306,7 +306,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C4" t="s">

</xml_diff>